<commit_message>
docs: add "Judge 2022 example" tab to the methodology workbook
Second worksheet walks through Aaron Judge's 2022 season value (+19.9) step by
step: the 6 categories in play that year, building the 153-hitter pool, scoring
counting cats vs the pool in standard deviations (HR in full), the playing-time
weighting for rate cats (OBP in full), summing to the value, what the number
means, how a standard deviation is computed on the HR pool (plus a by-hand
mini-example), and why the 20-AB minimum is where it is.

make_methodology_xlsx.pl now emits 2 sheets (4th cell style for sub-rows);
.ps1 zips the extra part. Same walkthrough appended to docs/methodology.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FantasyMags-Methodology.xlsx
+++ b/FantasyMags-Methodology.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Methodology" sheetId="1" r:id="rId1"/>
+    <sheet name="Judge 2022 example" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -18,6 +19,11 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -47,12 +53,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -897,7 +906,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FULL SEASON, regardless of owner or timing. Scored against THAT season's categories (OPS only from the year it was added, etc.). Source = ESPN end-of-season roster snapshot stat lines (complete back to 2008; no outside data). Counting cats (R,HR,RBI,SB,W,K,SV,HLD,IP): z-score of the raw total vs the pool. Rate cats (AVG,OBP,SLG,OPS,ERA,WHIP,K/9): playing-time weighted -- contribution = (player rate - pool PT-weighted rate) x playing time (AB / PA / IP), then z-scored; ERA &amp; WHIP flipped so lower is better. Pool = top (teams x starting slots x 1.6) at hitting and at pitching. ~0 = replacement-level regular; elite ~+10 to +19; no explicit replacement subtraction in v1. Two-way players valued on both sides. Needs ~20 AB or ~10 IP to be valued. In-progress seasons use the current year's to-date line.</t>
+          <t xml:space="preserve">FULL SEASON, regardless of owner or timing. Scored against THAT season's categories (OPS only from the year it was added, etc.). Source = ESPN end-of-season roster snapshot stat lines (complete back to 2008; no outside data). Counting cats (R,HR,RBI,SB,W,K,SV,HLD,IP): z-score of the raw total vs the pool. Rate cats (AVG,OBP,SLG,OPS,ERA,WHIP,K/9): playing-time weighted -- contribution = (player rate - pool PT-weighted rate) x playing time (AB / PA / IP), then z-scored; ERA &amp; WHIP flipped so lower is better. Pool = top (teams x starting slots x 1.6) at hitting and at pitching. ~0 = replacement-level regular; elite ~+10 to +19; no explicit replacement subtraction in v1. Two-way players valued on both sides. Needs ~20 AB or ~10 IP to be valued. In-progress seasons use the current year's to-date line.  See the "Judge 2022 example" tab for a full walkthrough.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -924,7 +933,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Each player-season is credited to the drafting manager; the card also shows who held him at season's end.</t>
+          <t xml:space="preserve">Each player-season is credited to the manager who drafted the player; the card also shows who held him at season's end.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1005,4 +1014,751 @@
   </sheetData>
   <autoFilter ref="A1:F29"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="95" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Aaron Judge - 2022 - how the +19.9 season value is built</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THE SHORT VERSION</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value = for each scoring category, how many standard deviations better than a typical rosterable hitter he was, added up. A "standard deviation" is just a normal amount of spread: if most rostered hitters are within about 10 HR of each other, 1 standard deviation is about 10 HR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STEP 1  -  which categories counted in 2022</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The FBL used 6 hitting categories that year: Runs, HR, RBI, SB, Slugging, On-Base %. Only hitting categories apply to a hitter; pitching categories are scored separately for pitchers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STEP 2  -  build the pool</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Take every hitter that season with about 20 or more at-bats (a real amount of playing time). In 2022 that is 153 hitters. This pool is the yardstick: "a typical rosterable hitter" means the average of this group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STEP 3  -  score the counting categories (Runs, HR, RBI, SB)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare his total to the pool, measured in standard deviations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home runs, worked in full:</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pool average</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18.9 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   1 standard deviation (typical spread)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9.8 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Judge</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Score</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(62 - 18.9) / 9.8 = +4.38   -&gt;   about 4.4 "normal gaps" above average</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All four counting categories:</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Runs</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judge 133  |  pool avg ~78  |  score +2.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   HR</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judge 62  |  pool avg ~19  |  score +4.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   RBI</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judge 131  |  pool avg ~74  |  score +2.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SB</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judge 16  |  pool avg ~13  |  score +0.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STEP 4  -  score the rate categories (SLG, OBP)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A .425 on-base in 25 at-bats is not as valuable as .425 over a full year, so rates are weighted by playing time. The question becomes: over all his plate appearances, how many EXTRA times did he reach base compared with an average hitter?</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On-base %, worked in full:</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Playing-time-weighted league OBP</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Judge OBP, over 696 plate appearances</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.425</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Extra times on base</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">696 x (.425 - .334) = about 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   1 standard deviation of that "extra times on base" number across the pool</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">about 16.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Score</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">63 / 16.6 = +3.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Slugging</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same method  -&gt;  +5.07 (a .686 slugging over a full season)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STEP 5  -  add it up</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Runs</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+2.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   HR</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+4.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   RBI</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+2.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SB</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+0.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   SLG</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+5.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   OBP</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+3.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   VALUE</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+19.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WHAT THE NUMBER MEANS</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   about 0</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">replacement-level everyday player - a waiver-wire stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   +8 to +12</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a strong first-round season</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   +19.9</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">best in league history: elite (not just good) in five of six categories in the same year; only SB is ordinary</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOW "1 STANDARD DEVIATION" IS CALCULATED  (the 2022 HR pool)</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step 1 - average</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2,885 total HR / 153 hitters = 18.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step 2 - distance from average, per hitter</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">their HR minus 18.86  (a 30-HR hitter is +11.1; Judge is +43.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step 3 - square each distance and add them up</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sum = 14,719   (squaring makes them all positive and weights big misses more)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step 4 - divide by (hitters - 1), then square-root</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14,719 / 152 = 96.8 (variance);   sqrt(96.8) = 9.84 (standard deviation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why square then square-root</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">raw distances would cancel to zero; the square-root at the end puts the answer back in home runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiny version you can check by hand</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 hitters: 8, 14, 19, 24, 30 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   mean</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">95 / 5 = 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   squared distances</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">121 + 25 + 0 + 25 + 121 = 292</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   variance, then standard deviation</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">292 / 4 = 73;   sqrt(73) = 8.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">THE 20 AT-BAT MINIMUM</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A judgment call, not a statistical rule. It only keeps cup-of-coffee seasons out of the list and the pool pre-rank. It is deliberately low because the rate-stat weighting and the counting-stat penalties already handle small samples on their own. Raising it (say to 50 AB) would drop marginal names but move no real player's value.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: methodology - Draft Grades now covers the baseball path
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FantasyMags-Methodology.xlsx
+++ b/FantasyMags-Methodology.xlsx
@@ -763,7 +763,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Draft Grades (football)</t>
+          <t xml:space="preserve">Draft Grades</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -778,12 +778,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">We grade the PICK not the management: outcome = drafted player's full-season points that year / that season's baseline (mean of the top half of drafted players). Dynasty rookie picks also get a draft-time grade from current trade value vs slot, only for classes with 0-1 completed seasons. Expected value by round = mean outcome at that round across all gradeable drafts, lightly smoothed. Pick weight = 1/sqrt(round). Letter is a curve: z-score of the manager's score vs all graded manager-drafts (A+ at ~1.3 SD). Keeper and auction drafts are skipped; future seasons show "TBD".</t>
+          <t xml:space="preserve">We grade the PICK not the management: outcome = drafted player's full-season points that year / that season's baseline (mean of the top half of drafted players). BASEBALL: outcome = the drafted player's season VALUE (category z-score sum from the Players tab); already era-adjusted, so no baseline division. Dynasty rookie picks also get a draft-time grade from current trade value vs slot, only for classes with 0-1 completed seasons. Expected value by round = mean outcome at that round across all gradeable drafts, lightly smoothed. Pick weight = 1/sqrt(round). Letter is a curve: z-score of the manager's score vs all graded manager-drafts (A+ at ~1.3 SD). Keeper and auction drafts skipped; a season still in progress (no champion yet) is withheld until it finishes; a pick whose player never cleared ~20 AB / ~10 IP that year has no value and is skipped.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2019: Ryan Lenahan took Christian McCaffrey at 1.02; CMC returned 1.2x baseline that year -&gt; large positive surplus -&gt; contributes to an A+ class.</t>
+          <t xml:space="preserve">2019 FBL: Carl Pashko took Trout 1.1, Cole 2.12 and Bellinger 4.12 -- three top-of-league values -&gt; A+ class. 2019 dynasty: Ryan Lenahan took CMC at 1.02, who returned 1.2x baseline that year -&gt; large positive surplus.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: methodology - Trade Calculator now covers the baseball path
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FantasyMags-Methodology.xlsx
+++ b/FantasyMags-Methodology.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trade Calculator (football)</t>
+          <t xml:space="preserve">Trade Calculator</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -805,17 +805,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sum the market value of each side's players and picks; show who the trade favors and by how much.</t>
+          <t xml:space="preserve">Sum the value of each side's players (and picks, football); show who the trade favors and by how much.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Player values are a build-time FantasyCalc snapshot matched to the league format (SF/1-QB, PPR, teams). Pick values use FantasyCalc generic tiers. Verdict: &lt;3% Even, &lt;8% Slight edge, &lt;20% Favors, else Lopsided. Favored side = whoever RECEIVES more value. Roster-crunch (on by default): if the sides trade an unequal number of PLAYERS (picks do not count), the side getting more players has its cheapest bench values added, since it must cut to fit them.</t>
+          <t xml:space="preserve">FOOTBALL: values are a build-time FantasyCalc snapshot matched to league format (SF/1-QB, PPR, teams); pick values use FantasyCalc generic tiers; roster-crunch (on by default) adds the cheapest bench values to the side receiving more players. BASEBALL: no external market -&gt; values are our own season value (category z-score sum); you pick a season (redraft rosters change yearly); a team's roster is its end-of-season roster that year; trade value = season value floored at 0; no roster-crunch, no intel report. Verdict both sports: &lt;3% Even, &lt;8% Slight edge, &lt;20% Favors, else Lopsided. Favored side = whoever RECEIVES more value.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A sends one player (1930); B sends two (2552 total) -&gt; "A wins by 622 (24%)". With crunch on, B also absorbs a body, shrinking the edge.</t>
+          <t xml:space="preserve">Baseball 2024: Lindor 6.9 + Teoscar 4.7 vs Juan Soto 10.2 -&gt; "Carl comes out ahead, 1.3 in value (12%)".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: methodology - reflect shipped thresholds (60-game floor, min-15 rivalries, active-only title chase)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FantasyMags-Methodology.xlsx
+++ b/FantasyMags-Methodology.xlsx
@@ -362,7 +362,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate metrics have a games floor: football 20 all-time / 24 combined / 4 playoff; baseball target 60 reg-season / 60 combined / none for playoffs. "Trades" ignores scope and is hidden when a league has no trade data. Manual seasons are excluded here.</t>
+          <t xml:space="preserve">Rate metrics have a games floor: football 20 all-time / 24 combined / 4 playoff; BASEBALL 60 regular / 60 combined / none for playoffs. "Trades" ignores scope and is hidden when a league has no trade data. Manual seasons are excluded here.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -426,7 +426,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A pairing needs a minimum number of meetings to list: currently 12, target 15 for the 24-year baseball league.</t>
+          <t xml:space="preserve">A pairing needs a minimum number of meetings to list: 12 for football, 15 for the 24-year baseball league.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">We grade the PICK not the management: outcome = drafted player's full-season points that year / that season's baseline (mean of the top half of drafted players). BASEBALL: outcome = the drafted player's season VALUE (category z-score sum from the Players tab); already era-adjusted, so no baseline division. Dynasty rookie picks also get a draft-time grade from current trade value vs slot, only for classes with 0-1 completed seasons. Expected value by round = mean outcome at that round across all gradeable drafts, lightly smoothed. Pick weight = 1/sqrt(round). Letter is a curve: z-score of the manager's score vs all graded manager-drafts (A+ at ~1.3 SD). Keeper and auction drafts skipped; a season still in progress (no champion yet) is withheld until it finishes; a pick whose player never cleared ~20 AB / ~10 IP that year has no value and is skipped.</t>
+          <t xml:space="preserve">We grade the PICK not the management: outcome = drafted player's full-season points that year / that season's baseline (mean of the top half of drafted players). BASEBALL: outcome = the drafted player's season VALUE (category z-score sum from the Players tab); already era-adjusted, so no baseline division. Dynasty rookie picks also get a draft-time grade from current trade value vs slot, only for classes with 0-1 completed seasons. Expected value by round = mean outcome at that round across all gradeable drafts, lightly smoothed. Pick weight = 1/sqrt(round). Letter is a curve: z-score of the manager's score vs all graded manager-drafts (A+ at ~1.3 SD). 12 for football, 15 (category leagues); keeper and auction drafts skipped; a season still in progress (no champion yet) is withheld until it finishes; a pick whose player never cleared ~20 AB / ~10 IP that year has no value and is skipped.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">

</xml_diff>